<commit_message>
Aminolab and app.py update
</commit_message>
<xml_diff>
--- a/df_summary.xlsx
+++ b/df_summary.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check1_1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check2_2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check3_3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check4_4" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check5_5" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check6_6" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check7_7" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="מי תהום - קו מאסף" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="מי תהום - קידוח הפקה 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="מי תהום - קידוח הפקה 4" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="מי תהום - קידוח הפקה 8" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="מי תהום - קידוח הפקה 01" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="מי תהום - קידוח הפקה 21" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="מי תהום - קידוח הפקה 61" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +23,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,23 +419,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>08:30 :העש ,10/08/2025</t>
         </is>
       </c>
     </row>
@@ -994,10 +987,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -1007,11 +1002,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1022,7 +1017,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1037,7 +1032,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1052,11 +1047,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1067,7 +1062,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1082,11 +1077,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1097,11 +1092,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1112,7 +1107,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1127,11 +1122,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1142,7 +1137,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1157,7 +1152,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1172,7 +1167,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1187,7 +1182,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1202,11 +1197,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1217,11 +1212,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1232,7 +1227,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1247,7 +1242,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1262,11 +1257,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1277,11 +1272,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1292,7 +1287,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1307,7 +1302,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1322,7 +1317,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1337,11 +1332,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1352,7 +1347,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1367,11 +1362,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1382,7 +1377,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1397,11 +1392,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1412,10 +1407,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -1425,10 +1422,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -1438,7 +1437,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1453,11 +1452,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1468,11 +1467,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1483,11 +1482,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1498,13 +1497,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -1521,23 +1640,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -2084,10 +2208,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -2097,11 +2223,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -2112,7 +2238,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2127,7 +2253,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2142,11 +2268,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -2157,7 +2283,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,11 +2298,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2187,11 +2313,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -2202,7 +2328,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -2217,11 +2343,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -2232,7 +2358,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -2247,7 +2373,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2262,7 +2388,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -2277,7 +2403,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2292,11 +2418,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -2307,11 +2433,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2322,7 +2448,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -2337,7 +2463,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2352,11 +2478,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2367,11 +2493,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2382,7 +2508,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2397,7 +2523,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2412,7 +2538,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2427,11 +2553,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2442,7 +2568,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2457,11 +2583,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2472,7 +2598,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2487,11 +2613,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2502,10 +2628,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -2515,10 +2643,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -2528,7 +2658,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2543,11 +2673,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2558,11 +2688,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2573,11 +2703,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2588,13 +2718,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -2611,23 +2861,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -3174,10 +3429,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -3187,11 +3444,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3202,7 +3459,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3217,7 +3474,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3232,11 +3489,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -3247,7 +3504,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3262,11 +3519,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -3277,11 +3534,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -3292,7 +3549,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3307,11 +3564,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -3322,7 +3579,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -3337,7 +3594,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -3352,7 +3609,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -3367,7 +3624,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -3382,11 +3639,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -3397,11 +3654,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -3412,7 +3669,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -3427,7 +3684,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -3442,11 +3699,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -3457,11 +3714,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -3472,7 +3729,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -3487,7 +3744,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -3502,7 +3759,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -3517,11 +3774,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -3532,7 +3789,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -3547,11 +3804,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -3562,7 +3819,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -3577,11 +3834,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -3592,10 +3849,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -3605,10 +3864,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -3618,7 +3879,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -3633,11 +3894,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -3648,11 +3909,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -3663,11 +3924,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -3678,13 +3939,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -3701,23 +4082,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -4264,10 +4650,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -4277,11 +4665,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4292,7 +4680,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -4307,7 +4695,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -4322,11 +4710,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -4337,7 +4725,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -4352,11 +4740,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -4367,11 +4755,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -4382,7 +4770,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -4397,11 +4785,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -4412,7 +4800,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -4427,7 +4815,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -4442,7 +4830,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -4457,7 +4845,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -4472,11 +4860,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -4487,11 +4875,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -4502,7 +4890,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -4517,7 +4905,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4532,11 +4920,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -4547,11 +4935,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -4562,7 +4950,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4577,7 +4965,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4592,7 +4980,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4607,11 +4995,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -4622,7 +5010,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4637,11 +5025,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -4652,7 +5040,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4667,11 +5055,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -4682,10 +5070,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -4695,10 +5085,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -4708,7 +5100,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -4723,11 +5115,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -4738,11 +5130,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -4753,11 +5145,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -4768,13 +5160,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -4791,23 +5303,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -5354,10 +5871,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -5367,11 +5886,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -5382,7 +5901,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -5397,7 +5916,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -5412,11 +5931,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -5427,7 +5946,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -5442,11 +5961,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -5457,11 +5976,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -5472,7 +5991,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -5487,11 +6006,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -5502,7 +6021,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -5517,7 +6036,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -5532,7 +6051,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -5547,7 +6066,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -5562,11 +6081,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -5577,11 +6096,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -5592,7 +6111,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -5607,7 +6126,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -5622,11 +6141,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -5637,11 +6156,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -5652,7 +6171,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -5667,7 +6186,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -5682,7 +6201,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -5697,11 +6216,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -5712,7 +6231,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -5727,11 +6246,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -5742,7 +6261,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -5757,11 +6276,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -5772,10 +6291,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -5785,10 +6306,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -5798,7 +6321,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -5813,11 +6336,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -5828,11 +6351,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -5843,11 +6366,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -5858,13 +6381,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -5881,23 +6524,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -6444,10 +7092,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -6457,11 +7107,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -6472,7 +7122,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -6487,7 +7137,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -6502,11 +7152,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -6517,7 +7167,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -6532,11 +7182,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -6547,11 +7197,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -6562,7 +7212,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -6577,11 +7227,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -6592,7 +7242,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -6607,7 +7257,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -6622,7 +7272,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -6637,7 +7287,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -6652,11 +7302,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -6667,11 +7317,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -6682,7 +7332,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -6697,7 +7347,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -6712,11 +7362,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -6727,11 +7377,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -6742,7 +7392,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -6757,7 +7407,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -6772,7 +7422,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -6787,11 +7437,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -6802,7 +7452,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -6817,11 +7467,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -6832,7 +7482,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6847,11 +7497,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -6862,10 +7512,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -6875,10 +7527,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -6888,7 +7542,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -6903,11 +7557,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -6918,11 +7572,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -6933,11 +7587,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -6948,13 +7602,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>
@@ -6971,23 +7745,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>units</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>10/08/2025</t>
         </is>
       </c>
     </row>
@@ -7534,10 +8313,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>Trichloroethane</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -7547,11 +8328,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Toluene</t>
+          <t>Trichloroethane</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -7562,7 +8343,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>transDichloroethene</t>
+          <t>Dichloroethane</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -7577,7 +8358,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>transDichloropropene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -7592,11 +8373,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Trichloroethene</t>
+          <t>Trichlorobenzene</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -7607,7 +8388,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dichloropropene</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -7622,11 +8403,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>tetrachlorethane</t>
+          <t>DibromoethaneEthylenedibromide</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -7637,11 +8418,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tetrachloroethane</t>
+          <t>Dichloropropane</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -7652,7 +8433,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trichloropropane</t>
+          <t>Trimethylbenzene</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -7667,11 +8448,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dibromochloropropane</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -7682,7 +8463,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Bromodichloromethane</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -7697,7 +8478,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dichlorobenzene</t>
+          <t>Toluene</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -7712,7 +8493,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dichloropropane</t>
+          <t>transDichloroethene</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -7727,7 +8508,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>transDichloropropene</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -7742,11 +8523,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chlorotoluene</t>
+          <t>Trichloroethene</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -7757,11 +8538,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Benzene</t>
+          <t>Dichloropropene</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -7772,7 +8553,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bromobenzene</t>
+          <t>tetrachlorethane</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -7787,7 +8568,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bromochloromethan</t>
+          <t>Tetrachloroethane</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -7802,11 +8583,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Carbontetrachloride</t>
+          <t>Trichloropropane</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -7817,11 +8598,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chloroethane</t>
+          <t>Dibromochloropropane</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -7832,7 +8613,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chloroform</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -7847,7 +8628,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cisDichloroethene</t>
+          <t>Dichlorobenzene</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -7862,7 +8643,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Methanechloro</t>
+          <t>dichloropropane</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -7877,11 +8658,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MTBE</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -7892,7 +8673,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mXylene</t>
+          <t>Chlorotoluene</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -7907,11 +8688,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pIsopropyltoluene</t>
+          <t>Benzene</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -7922,7 +8703,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Styrene</t>
+          <t>Bromobenzene</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -7937,11 +8718,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinylchloride</t>
+          <t>Bromochloromethan</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -7952,10 +8733,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>חתימה</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
+          <t>Carbontetrachloride</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -7965,10 +8748,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Compound</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
+          <t>Chloroethane</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>5</v>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>ppb</t>
@@ -7978,7 +8763,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>oxylene</t>
+          <t>Chloroform</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -7993,11 +8778,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dichloroethylene</t>
+          <t>cisDichloroethene</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -8008,11 +8793,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tetrachloroethene</t>
+          <t>Methanechloro</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -8023,11 +8808,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dichloroethane</t>
+          <t>MTBE</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -8038,13 +8823,133 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>mXylene</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>pIsopropyltoluene</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Styrene</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vinylchloride</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>oxylene</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Dichloroethylene</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tetrachloroethene</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Dichloroethane</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>pXylene</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>5</v>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B80" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>ppb</t>
         </is>

</xml_diff>